<commit_message>
correct expected return calc to account for calendar days
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64E769AE-D343-4D7A-BF8C-60F6E05796B9}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A3D7997-AB1E-4A98-8D0F-C79DE25411F3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
-    <sheet name="Dates &amp;amp;amp;amp;amp;amp; Ris" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,16 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>End Date</t>
-  </si>
-  <si>
-    <t>Risk Free Rate</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Ticker</t>
   </si>
@@ -91,8 +81,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.00%"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="#,##0%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
@@ -137,26 +126,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -474,218 +445,144 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="8">
-        <v>0</v>
-      </c>
-      <c r="C2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F2" s="8">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="8">
-        <v>0</v>
-      </c>
-      <c r="C3" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F3" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="8">
-        <v>0</v>
-      </c>
-      <c r="C4" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F4" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="8">
-        <v>0</v>
-      </c>
-      <c r="C5" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F5" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F6" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="8">
-        <v>0</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="8">
-        <v>0</v>
-      </c>
-      <c r="C8" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F8" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="8">
-        <v>0</v>
-      </c>
-      <c r="C9" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F9" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="8">
-        <v>0</v>
-      </c>
-      <c r="C10" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F10" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="8">
-        <v>0</v>
-      </c>
-      <c r="C11" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="F11" s="8">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="10">
-        <v>0</v>
-      </c>
-      <c r="C12" s="8">
-        <v>0.02</v>
-      </c>
-      <c r="F12" s="8">
-        <v>0.02</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="2" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" style="6" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
-        <f ca="1">DATE(YEAR(B2)-10,MONTH(B2),DAY(B2))</f>
-        <v>41864</v>
-      </c>
-      <c r="B2" s="3">
-        <f ca="1">NOW()</f>
-        <v>45517.659255324077</v>
-      </c>
-      <c r="C2" s="4">
-        <v>5.1499999999999997E-2</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added return & risk for +/- 1 & 2 std Dev
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A3D7997-AB1E-4A98-8D0F-C79DE25411F3}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4297A59-4185-4841-A1C4-1F7106A3B71C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="#,##0%"/>
+    <numFmt numFmtId="164" formatCode="#,##0%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -128,16 +128,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -155,6 +155,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -472,7 +476,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="2">
-        <v>0.5</v>
+        <v>0.99999000000000005</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -538,7 +542,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="2">
-        <v>0.6</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -549,7 +553,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="2">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -560,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="2">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -582,7 +586,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated asset_classes excel sheets
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4297A59-4185-4841-A1C4-1F7106A3B71C}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F6F0DC-6128-42E4-9205-6C6CA111722A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -155,10 +155,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -586,7 +582,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add "Curr Weight" field to Excel sheets. Check that sum of "Max Weight" is >= 100%.
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F6F0DC-6128-42E4-9205-6C6CA111722A}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB222890-6A0E-4B20-9640-7C8A884728BE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Ticker</t>
   </si>
@@ -75,14 +75,18 @@
   </si>
   <si>
     <t>IAU</t>
+  </si>
+  <si>
+    <t>Curr Weight</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -126,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -138,6 +142,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -445,7 +455,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
@@ -453,7 +463,7 @@
     <col min="3" max="3" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -463,8 +473,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -474,8 +487,12 @@
       <c r="C2" s="2">
         <v>0.99999000000000005</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2" s="6">
+        <f>1/11</f>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -485,8 +502,12 @@
       <c r="C3" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" s="6">
+        <f t="shared" ref="D3:D12" si="0">1/11</f>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -496,8 +517,12 @@
       <c r="C4" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -507,8 +532,12 @@
       <c r="C5" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -518,8 +547,12 @@
       <c r="C6" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -529,8 +562,12 @@
       <c r="C7" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -540,8 +577,12 @@
       <c r="C8" s="2">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -551,8 +592,12 @@
       <c r="C9" s="2">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -562,8 +607,12 @@
       <c r="C10" s="2">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -573,8 +622,12 @@
       <c r="C11" s="2">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -583,6 +636,10 @@
       </c>
       <c r="C12" s="2">
         <v>0.03</v>
+      </c>
+      <c r="D12" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add comparison of current vs selected portfolios
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB222890-6A0E-4B20-9640-7C8A884728BE}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59B3FFCD-82BF-4E2A-A82A-C52CEDF77885}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40" yWindow="0" windowWidth="25560" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
@@ -86,7 +86,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00%"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -147,7 +147,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -461,6 +461,7 @@
     <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.453125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -488,8 +489,7 @@
         <v>0.99999000000000005</v>
       </c>
       <c r="D2" s="6">
-        <f>1/11</f>
-        <v>9.0909090909090912E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -503,8 +503,8 @@
         <v>0.6</v>
       </c>
       <c r="D3" s="6">
-        <f t="shared" ref="D3:D12" si="0">1/11</f>
-        <v>9.0909090909090912E-2</v>
+        <f>0.1/4</f>
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -518,8 +518,8 @@
         <v>0.6</v>
       </c>
       <c r="D4" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <f t="shared" ref="D4:D6" si="0">0.1/4</f>
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" s="6">
         <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -549,7 +549,7 @@
       </c>
       <c r="D6" s="6">
         <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -563,8 +563,7 @@
         <v>0.6</v>
       </c>
       <c r="D7" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -578,8 +577,7 @@
         <v>0.25</v>
       </c>
       <c r="D8" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -593,8 +591,8 @@
         <v>0.2</v>
       </c>
       <c r="D9" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <f>0.22*(2/3)</f>
+        <v>0.14666666666666667</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -608,8 +606,8 @@
         <v>0.1</v>
       </c>
       <c r="D10" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <f>0.22*(1/3)</f>
+        <v>7.3333333333333334E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -623,8 +621,7 @@
         <v>0.05</v>
       </c>
       <c r="D11" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -635,11 +632,10 @@
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="D12" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added Instructions, Links to Helpful Info, & Tool Tips. Revised fmc.xlsx
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59B3FFCD-82BF-4E2A-A82A-C52CEDF77885}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8458A9D-EA08-444E-933A-95079807FB68}"/>
   <bookViews>
     <workbookView xWindow="40" yWindow="0" windowWidth="25560" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,9 +488,7 @@
       <c r="C2" s="2">
         <v>0.99999000000000005</v>
       </c>
-      <c r="D2" s="6">
-        <v>0</v>
-      </c>
+      <c r="D2" s="6"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -502,10 +500,7 @@
       <c r="C3" s="2">
         <v>0.6</v>
       </c>
-      <c r="D3" s="6">
-        <f>0.1/4</f>
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -517,10 +512,7 @@
       <c r="C4" s="2">
         <v>0.6</v>
       </c>
-      <c r="D4" s="6">
-        <f t="shared" ref="D4:D6" si="0">0.1/4</f>
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="D4" s="6"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -532,10 +524,7 @@
       <c r="C5" s="2">
         <v>0.6</v>
       </c>
-      <c r="D5" s="6">
-        <f t="shared" si="0"/>
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -547,10 +536,7 @@
       <c r="C6" s="2">
         <v>0.6</v>
       </c>
-      <c r="D6" s="6">
-        <f t="shared" si="0"/>
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -562,9 +548,7 @@
       <c r="C7" s="2">
         <v>0.6</v>
       </c>
-      <c r="D7" s="6">
-        <v>0.47</v>
-      </c>
+      <c r="D7" s="6"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -576,9 +560,7 @@
       <c r="C8" s="2">
         <v>0.25</v>
       </c>
-      <c r="D8" s="6">
-        <v>0.16</v>
-      </c>
+      <c r="D8" s="6"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -590,10 +572,7 @@
       <c r="C9" s="2">
         <v>0.2</v>
       </c>
-      <c r="D9" s="6">
-        <f>0.22*(2/3)</f>
-        <v>0.14666666666666667</v>
-      </c>
+      <c r="D9" s="6"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -605,10 +584,7 @@
       <c r="C10" s="2">
         <v>0.1</v>
       </c>
-      <c r="D10" s="6">
-        <f>0.22*(1/3)</f>
-        <v>7.3333333333333334E-2</v>
-      </c>
+      <c r="D10" s="6"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -620,9 +596,7 @@
       <c r="C11" s="2">
         <v>0.05</v>
       </c>
-      <c r="D11" s="6">
-        <v>0.05</v>
-      </c>
+      <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -634,9 +608,7 @@
       <c r="C12" s="2">
         <v>0</v>
       </c>
-      <c r="D12" s="6">
-        <v>0</v>
-      </c>
+      <c r="D12" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
minor spelling & grammer
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained.xlsx
+++ b/data/asset_classes_constrained.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8458A9D-EA08-444E-933A-95079807FB68}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{C00631DB-D9B0-4189-947F-2BB70603FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46563C57-DCB1-48AA-8055-128938BAB59D}"/>
   <bookViews>
-    <workbookView xWindow="40" yWindow="0" windowWidth="25560" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="D12" s="6"/>
     </row>

</xml_diff>